<commit_message>
Umstrukturierung und Hochladen alles bisher
</commit_message>
<xml_diff>
--- a/Kosten.xlsx
+++ b/Kosten.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\HTL_Anichstrasse\Werkstaette\R6_Drone\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\HTL_Anichstrasse\Werkstaette\R6_Drone_nogit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96A39AFE-150F-4721-8052-D43A9349E913}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCB91909-92F5-432A-9340-A85A1C5553B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6DD5FD97-CAD3-4E1A-A256-A5B1796696A9}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="28">
   <si>
     <t>Bauteil</t>
   </si>
@@ -62,33 +62,21 @@
     <t>OV2640 160° kamera</t>
   </si>
   <si>
-    <t>INMP441 Mikrofon</t>
-  </si>
-  <si>
     <t>A4988 Stepperdriver</t>
   </si>
   <si>
     <t>NEMA 17 Steppermotor</t>
   </si>
   <si>
-    <t>Stück gekauft</t>
-  </si>
-  <si>
     <t>Tatsächliche Ausgaben</t>
   </si>
   <si>
-    <t>Kosten pro Drohne + Controller</t>
-  </si>
-  <si>
     <t>Mekanumräder</t>
   </si>
   <si>
     <t>?</t>
   </si>
   <si>
-    <t>Buck-Converter</t>
-  </si>
-  <si>
     <t>RGB Streifen (10cm)</t>
   </si>
   <si>
@@ -101,7 +89,37 @@
     <t>PS4 Controller</t>
   </si>
   <si>
-    <t>Multi-Akku-Ladegeräat</t>
+    <t>100nF Keramik-Kondensatoren</t>
+  </si>
+  <si>
+    <t>Bestellungen</t>
+  </si>
+  <si>
+    <t>TSR-0-5-2450</t>
+  </si>
+  <si>
+    <t>100uF ELKO</t>
+  </si>
+  <si>
+    <t>theoretische Kosten pro Drohne + Controller</t>
+  </si>
+  <si>
+    <t>Multi-Akku-Ladegerät</t>
+  </si>
+  <si>
+    <t>Schraubklemmen 1x2</t>
+  </si>
+  <si>
+    <t>Loot:</t>
+  </si>
+  <si>
+    <t>ESP32-C3 Super Mini</t>
+  </si>
+  <si>
+    <t>ESP32-C3</t>
+  </si>
+  <si>
+    <t>Gyro-Sensor</t>
   </si>
 </sst>
 </file>
@@ -145,7 +163,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -188,8 +206,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -265,11 +289,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="7" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
@@ -301,9 +334,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -341,7 +371,28 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -676,15 +727,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5850C87B-A7EA-4251-8D17-A69A75D7F344}">
-  <dimension ref="B2:K15"/>
+  <dimension ref="B2:K22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.88671875" customWidth="1"/>
-    <col min="3" max="3" width="24.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20.44140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="29.6640625" customWidth="1"/>
+    <col min="7" max="7" width="37.33203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.77734375" customWidth="1"/>
     <col min="9" max="9" width="11.5546875" customWidth="1"/>
     <col min="10" max="10" width="14.21875" customWidth="1"/>
@@ -705,17 +756,17 @@
         <v>6</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" s="25" t="s">
-        <v>18</v>
+        <v>21</v>
+      </c>
+      <c r="H2" s="24" t="s">
+        <v>14</v>
       </c>
       <c r="I2" s="3"/>
       <c r="J2" s="5" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="K2" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
@@ -738,12 +789,12 @@
         <f>D3*E3</f>
         <v>11.09</v>
       </c>
-      <c r="H3" s="26"/>
+      <c r="H3" s="25"/>
       <c r="J3" s="8">
         <v>1</v>
       </c>
       <c r="K3" s="11">
-        <f t="shared" ref="K3:K12" si="0">E3*J3</f>
+        <f>F3*J3</f>
         <v>11.09</v>
       </c>
     </row>
@@ -765,99 +816,95 @@
         <f>D4*E4</f>
         <v>8</v>
       </c>
-      <c r="H4" s="26"/>
+      <c r="H4" s="25"/>
       <c r="J4" s="12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K4" s="15">
-        <f t="shared" si="0"/>
+        <f>F4*J4</f>
         <v>16</v>
       </c>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.3">
       <c r="C5" s="8" t="s">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="D5" s="9">
-        <v>1</v>
-      </c>
-      <c r="E5" s="10">
-        <f>13.1/5</f>
-        <v>2.62</v>
-      </c>
-      <c r="F5" s="10">
-        <v>13.1</v>
-      </c>
-      <c r="G5" s="11">
-        <f t="shared" ref="G5:G9" si="1">D5*E5</f>
-        <v>2.62</v>
-      </c>
-      <c r="H5" s="26"/>
+        <v>3</v>
+      </c>
+      <c r="E5" s="29" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="29" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" s="30" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5" s="25"/>
       <c r="J5" s="8">
-        <v>5</v>
-      </c>
-      <c r="K5" s="11">
-        <f t="shared" si="0"/>
-        <v>13.100000000000001</v>
+        <v>0</v>
+      </c>
+      <c r="K5" s="30" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.3">
       <c r="C6" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="21">
-        <v>1</v>
-      </c>
-      <c r="E6" s="22">
+        <v>13</v>
+      </c>
+      <c r="D6" s="20">
+        <v>1</v>
+      </c>
+      <c r="E6" s="21">
         <f>13.1/10</f>
         <v>1.31</v>
       </c>
-      <c r="F6" s="22">
+      <c r="F6" s="21">
         <v>13.1</v>
       </c>
-      <c r="G6" s="23">
-        <f t="shared" si="1"/>
+      <c r="G6" s="22">
+        <f t="shared" ref="G6:G9" si="0">D6*E6</f>
         <v>1.31</v>
       </c>
-      <c r="H6" s="26"/>
-      <c r="J6" s="24">
+      <c r="H6" s="25"/>
+      <c r="J6" s="23">
         <v>0</v>
       </c>
-      <c r="K6" s="23">
-        <f t="shared" si="0"/>
+      <c r="K6" s="15">
+        <f>F6*J6</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.3">
       <c r="C7" s="8" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D7" s="9">
         <v>1</v>
       </c>
       <c r="E7" s="10">
-        <f>9.56/5</f>
-        <v>1.9120000000000001</v>
+        <v>6</v>
       </c>
       <c r="F7" s="10">
-        <v>9.56</v>
+        <v>6</v>
       </c>
       <c r="G7" s="11">
-        <f t="shared" si="1"/>
-        <v>1.9120000000000001</v>
-      </c>
-      <c r="H7" s="26"/>
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="H7" s="25"/>
       <c r="J7" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K7" s="11">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>F7*J7</f>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.3">
       <c r="C8" s="12" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D8" s="13">
         <v>2</v>
@@ -873,18 +920,18 @@
         <f>D8*E8</f>
         <v>3.22</v>
       </c>
-      <c r="H8" s="26"/>
+      <c r="H8" s="25"/>
       <c r="J8" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K8" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>F8*J8</f>
+        <v>8.0500000000000007</v>
       </c>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.3">
       <c r="C9" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D9" s="9">
         <v>2</v>
@@ -896,73 +943,73 @@
         <v>14.11</v>
       </c>
       <c r="G9" s="11">
-        <f t="shared" si="1"/>
-        <v>28.22</v>
-      </c>
-      <c r="H9" s="26"/>
-      <c r="J9" s="8">
-        <v>2</v>
-      </c>
-      <c r="K9" s="11">
         <f t="shared" si="0"/>
         <v>28.22</v>
       </c>
+      <c r="H9" s="25"/>
+      <c r="J9" s="8">
+        <v>1</v>
+      </c>
+      <c r="K9" s="11">
+        <f>F9*J9</f>
+        <v>14.11</v>
+      </c>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.3">
       <c r="C10" s="12" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D10" s="13">
         <v>2</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="G10" s="20" t="s">
-        <v>15</v>
-      </c>
-      <c r="H10" s="27"/>
+        <v>12</v>
+      </c>
+      <c r="G10" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="H10" s="26"/>
       <c r="I10" s="3"/>
-      <c r="J10" s="24">
+      <c r="J10" s="23">
         <v>0</v>
       </c>
       <c r="K10" s="19" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.3">
       <c r="C11" s="1" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D11" s="2">
         <v>1</v>
       </c>
-      <c r="E11" s="32">
+      <c r="E11" s="31">
         <f>39/2</f>
         <v>19.5</v>
       </c>
-      <c r="F11" s="28">
+      <c r="F11" s="27">
         <v>39</v>
       </c>
-      <c r="G11" s="29">
+      <c r="G11" s="28">
         <v>19.5</v>
       </c>
-      <c r="H11" s="26"/>
+      <c r="H11" s="25"/>
       <c r="I11" s="3"/>
-      <c r="J11" s="33">
-        <v>2</v>
+      <c r="J11" s="32">
+        <v>1</v>
       </c>
       <c r="K11" s="11">
-        <f t="shared" si="0"/>
+        <f>F11*J11</f>
         <v>39</v>
       </c>
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.3">
       <c r="C12" s="12" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D12" s="13">
         <v>1</v>
@@ -976,59 +1023,188 @@
       <c r="G12" s="14">
         <v>34</v>
       </c>
-      <c r="H12" s="26"/>
+      <c r="H12" s="25"/>
       <c r="I12" s="3"/>
-      <c r="J12" s="34">
-        <v>1</v>
-      </c>
-      <c r="K12" s="35">
-        <f>E12*J12</f>
+      <c r="J12" s="33">
+        <v>1</v>
+      </c>
+      <c r="K12" s="34">
+        <f>F12*J12</f>
         <v>34</v>
       </c>
     </row>
-    <row r="14" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B14" s="4" t="s">
+    <row r="13" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="C13" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="2">
+        <v>3</v>
+      </c>
+      <c r="E13" s="35" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="36" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" s="37" t="s">
+        <v>12</v>
+      </c>
+      <c r="H13" s="25"/>
+      <c r="J13" s="32">
+        <v>0</v>
+      </c>
+      <c r="K13" s="38" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="C14" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D14" s="13">
+        <v>3</v>
+      </c>
+      <c r="E14" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="G14" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="H14" s="25"/>
+      <c r="J14" s="23">
+        <v>0</v>
+      </c>
+      <c r="K14" s="19" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="C15" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D15" s="2">
+        <v>1</v>
+      </c>
+      <c r="E15" s="35" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" s="36" t="s">
+        <v>12</v>
+      </c>
+      <c r="G15" s="37" t="s">
+        <v>12</v>
+      </c>
+      <c r="H15" s="43"/>
+      <c r="J15" s="32">
+        <v>0</v>
+      </c>
+      <c r="K15" s="38" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="C16" s="41" t="s">
+        <v>27</v>
+      </c>
+      <c r="D16" s="42">
+        <v>1</v>
+      </c>
+      <c r="E16" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="F16" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="G16" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="H16" s="25"/>
+      <c r="J16" s="23">
+        <v>0</v>
+      </c>
+      <c r="K16" s="19" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B18" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C14" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D14" s="9">
-        <v>1</v>
-      </c>
-      <c r="E14" s="30" t="s">
-        <v>15</v>
-      </c>
-      <c r="F14" s="30" t="s">
-        <v>15</v>
-      </c>
-      <c r="G14" s="30" t="s">
-        <v>15</v>
-      </c>
-      <c r="H14" s="26"/>
-      <c r="J14" s="8">
+      <c r="C18" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D18" s="9">
+        <v>1</v>
+      </c>
+      <c r="E18" s="29" t="s">
+        <v>12</v>
+      </c>
+      <c r="F18" s="29" t="s">
+        <v>12</v>
+      </c>
+      <c r="G18" s="29" t="s">
+        <v>12</v>
+      </c>
+      <c r="H18" s="25"/>
+      <c r="J18" s="8">
         <v>0</v>
       </c>
-      <c r="K14" s="31" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="15" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="C15" s="1"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="17">
-        <f>SUM(F3:F14)</f>
-        <v>158.01</v>
-      </c>
-      <c r="G15" s="16">
-        <f>SUM(G3:G14)</f>
-        <v>109.872</v>
-      </c>
-      <c r="J15" s="1"/>
-      <c r="K15" s="17">
-        <f>SUM(K3:K14)</f>
-        <v>141.41</v>
+      <c r="K18" s="30" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="C19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D19">
+        <v>1</v>
+      </c>
+      <c r="E19" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="F19" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="G19" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="H19" s="25"/>
+      <c r="J19">
+        <v>0</v>
+      </c>
+      <c r="K19" s="19" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="C20" s="1"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="17">
+        <f>SUM(F3:F18)</f>
+        <v>141.35</v>
+      </c>
+      <c r="G20" s="16">
+        <f>SUM(G3:G18)</f>
+        <v>111.34</v>
+      </c>
+      <c r="J20" s="1"/>
+      <c r="K20" s="17">
+        <f>SUM(K3:K18)</f>
+        <v>128.25</v>
+      </c>
+    </row>
+    <row r="22" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="J22" s="39" t="s">
+        <v>24</v>
+      </c>
+      <c r="K22" s="40">
+        <f>F20-K20</f>
+        <v>13.099999999999994</v>
       </c>
     </row>
   </sheetData>

</xml_diff>